<commit_message>
Reflect latest tracker updates
</commit_message>
<xml_diff>
--- a/public/data/RPA_Project_Tracker_Web_Ready.xlsx
+++ b/public/data/RPA_Project_Tracker_Web_Ready.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\KhalidAlharbi\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbookpro/Desktop/Rac For Project Tracker /Weekly update/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4EE40E6-6516-40E2-8B9D-F73DFDE5D167}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{992DBAC3-6D0F-0940-A8BD-1A52D3C84363}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="33600" windowHeight="21000" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="4" r:id="rId1"/>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1517" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1550" uniqueCount="192">
   <si>
     <t>Process / Phase</t>
   </si>
@@ -582,15 +582,56 @@
   </si>
   <si>
     <t>ROI</t>
+  </si>
+  <si>
+    <t>RAC - Ibrahim Al osaimi</t>
+  </si>
+  <si>
+    <t>The access was working for a while, but it has stopped working again.</t>
+  </si>
+  <si>
+    <t>Cyber Security Team</t>
+  </si>
+  <si>
+    <t>Abdulmohsen Abushaiqa</t>
+  </si>
+  <si>
+    <t>ICT</t>
+  </si>
+  <si>
+    <t>Abdulaziz Alodhibi</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>RITM0078287</t>
+  </si>
+  <si>
+    <t>Proven - Mohammed Shalaby</t>
+  </si>
+  <si>
+    <t>Mohammed Shalaby</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Ibrahim Al osaimi</t>
+  </si>
+  <si>
+    <t>Open a Policy Exception ticket, or provide us with the method to access the platform.</t>
+  </si>
+  <si>
+    <t>We cannot complete the setup until access to the platform is granted.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
-    <numFmt numFmtId="165" formatCode="dd\-mmm\-yyyy\ hh:mm"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="dd\-mmm\-yyyy\ hh:mm"/>
   </numFmts>
   <fonts count="27">
     <font>
@@ -738,16 +779,19 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF17365D"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF1F2937"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="19">
@@ -991,7 +1035,7 @@
   <cellXfs count="109">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1002,7 +1046,7 @@
     <xf numFmtId="0" fontId="20" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="21" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="22" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="3" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="14" fontId="3" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1020,7 +1064,7 @@
     <xf numFmtId="9" fontId="3" fillId="11" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="11" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="3" fillId="11" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1029,16 +1073,16 @@
     <xf numFmtId="9" fontId="0" fillId="10" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="10" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="0" fillId="10" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="7" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="6" fillId="7" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -1047,10 +1091,10 @@
     <xf numFmtId="0" fontId="0" fillId="12" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="12" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="0" fillId="12" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="12" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="5" fillId="12" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="16" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1074,7 +1118,7 @@
     <xf numFmtId="0" fontId="25" fillId="13" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="25" fillId="13" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="25" fillId="13" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1083,7 +1127,7 @@
     <xf numFmtId="0" fontId="26" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="26" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="26" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="14" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1104,10 +1148,95 @@
     <xf numFmtId="0" fontId="24" fillId="18" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="12" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="3" fillId="12" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="3" fillId="11" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="16" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="16" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="16" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="16" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="16" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="16" fillId="9" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="13" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="13" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="13" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="13" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="13" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="13" fillId="9" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="14" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="14" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="14" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="14" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="14" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="14" fillId="9" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="15" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="15" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="15" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="15" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="15" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="15" fillId="9" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1195,91 +1324,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="12" fillId="9" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="16" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="16" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="16" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="16" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="16" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="16" fillId="9" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="13" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="13" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="13" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="13" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="13" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="13" fillId="9" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="14" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="14" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="14" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="14" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="14" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="14" fillId="9" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="15" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="15" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="15" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="15" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="15" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="15" fillId="9" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1457,7 +1501,6 @@
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <xxl21:alternateUrls>
       <xxl21:absoluteUrl r:id="rId2"/>
-      <xxl21:relativeUrl r:id="rId3"/>
     </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Dashboard"/>
@@ -1715,7 +1758,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:O37"/>
-  <sheetFormatPr defaultRowHeight="14"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="3" width="12" customWidth="1"/>
@@ -1727,37 +1770,37 @@
     <col min="14" max="15" width="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="14.65" customHeight="1">
-      <c r="A1" s="49" t="s">
+    <row r="1" spans="1:15" ht="14.75" customHeight="1">
+      <c r="A1" s="78" t="s">
         <v>73</v>
       </c>
-      <c r="B1" s="49"/>
-      <c r="C1" s="49"/>
-      <c r="D1" s="49"/>
-      <c r="E1" s="49"/>
-      <c r="F1" s="49"/>
-      <c r="G1" s="49"/>
-      <c r="H1" s="49"/>
-      <c r="I1" s="49"/>
-      <c r="J1" s="49"/>
-      <c r="K1" s="49"/>
-      <c r="L1" s="49"/>
+      <c r="B1" s="78"/>
+      <c r="C1" s="78"/>
+      <c r="D1" s="78"/>
+      <c r="E1" s="78"/>
+      <c r="F1" s="78"/>
+      <c r="G1" s="78"/>
+      <c r="H1" s="78"/>
+      <c r="I1" s="78"/>
+      <c r="J1" s="78"/>
+      <c r="K1" s="78"/>
+      <c r="L1" s="78"/>
       <c r="N1" s="13"/>
       <c r="O1" s="13"/>
     </row>
-    <row r="2" spans="1:15" ht="14.65" customHeight="1">
-      <c r="A2" s="49"/>
-      <c r="B2" s="49"/>
-      <c r="C2" s="49"/>
-      <c r="D2" s="49"/>
-      <c r="E2" s="49"/>
-      <c r="F2" s="49"/>
-      <c r="G2" s="49"/>
-      <c r="H2" s="49"/>
-      <c r="I2" s="49"/>
-      <c r="J2" s="49"/>
-      <c r="K2" s="49"/>
-      <c r="L2" s="49"/>
+    <row r="2" spans="1:15" ht="14.75" customHeight="1">
+      <c r="A2" s="78"/>
+      <c r="B2" s="78"/>
+      <c r="C2" s="78"/>
+      <c r="D2" s="78"/>
+      <c r="E2" s="78"/>
+      <c r="F2" s="78"/>
+      <c r="G2" s="78"/>
+      <c r="H2" s="78"/>
+      <c r="I2" s="78"/>
+      <c r="J2" s="78"/>
+      <c r="K2" s="78"/>
+      <c r="L2" s="78"/>
       <c r="N2" s="13" t="s">
         <v>70</v>
       </c>
@@ -1765,22 +1808,22 @@
         <v>74</v>
       </c>
     </row>
-    <row r="3" spans="1:15" ht="14.65" customHeight="1">
-      <c r="A3" s="50" t="str">
+    <row r="3" spans="1:15" ht="14.75" customHeight="1">
+      <c r="A3" s="79" t="str">
         <f ca="1">"Updated: "&amp;TEXT(TODAY(),"dd/mm/yyyy")</f>
-        <v>Updated: 30/07/2026</v>
-      </c>
-      <c r="B3" s="50"/>
-      <c r="C3" s="50"/>
-      <c r="D3" s="50"/>
-      <c r="E3" s="50"/>
-      <c r="F3" s="50"/>
-      <c r="G3" s="50"/>
-      <c r="H3" s="50"/>
-      <c r="I3" s="50"/>
-      <c r="J3" s="50"/>
-      <c r="K3" s="50"/>
-      <c r="L3" s="50"/>
+        <v>Updated: 01/08/2026</v>
+      </c>
+      <c r="B3" s="79"/>
+      <c r="C3" s="79"/>
+      <c r="D3" s="79"/>
+      <c r="E3" s="79"/>
+      <c r="F3" s="79"/>
+      <c r="G3" s="79"/>
+      <c r="H3" s="79"/>
+      <c r="I3" s="79"/>
+      <c r="J3" s="79"/>
+      <c r="K3" s="79"/>
+      <c r="L3" s="79"/>
       <c r="N3" s="13" t="s">
         <v>58</v>
       </c>
@@ -1789,7 +1832,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:15" ht="14.65" customHeight="1">
+    <row r="4" spans="1:15" ht="14.75" customHeight="1">
       <c r="A4" s="3"/>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
@@ -1810,27 +1853,27 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:15" ht="14.65" customHeight="1">
-      <c r="A5" s="51" t="s">
+    <row r="5" spans="1:15" ht="14.75" customHeight="1">
+      <c r="A5" s="80" t="s">
         <v>75</v>
       </c>
-      <c r="B5" s="51"/>
-      <c r="C5" s="51"/>
-      <c r="D5" s="51" t="s">
+      <c r="B5" s="80"/>
+      <c r="C5" s="80"/>
+      <c r="D5" s="80" t="s">
         <v>76</v>
       </c>
-      <c r="E5" s="51"/>
-      <c r="F5" s="51"/>
-      <c r="G5" s="64" t="s">
+      <c r="E5" s="80"/>
+      <c r="F5" s="80"/>
+      <c r="G5" s="93" t="s">
         <v>77</v>
       </c>
-      <c r="H5" s="64"/>
-      <c r="I5" s="64"/>
-      <c r="J5" s="71" t="s">
+      <c r="H5" s="93"/>
+      <c r="I5" s="93"/>
+      <c r="J5" s="100" t="s">
         <v>78</v>
       </c>
-      <c r="K5" s="71"/>
-      <c r="L5" s="71"/>
+      <c r="K5" s="100"/>
+      <c r="L5" s="100"/>
       <c r="N5" s="13" t="s">
         <v>11</v>
       </c>
@@ -1839,31 +1882,31 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:15" ht="14.65" customHeight="1">
-      <c r="A6" s="52">
+    <row r="6" spans="1:15" ht="14.75" customHeight="1">
+      <c r="A6" s="81">
         <f>COUNTA('Process Summary'!A4:A33)</f>
         <v>30</v>
       </c>
-      <c r="B6" s="53"/>
-      <c r="C6" s="54"/>
-      <c r="D6" s="58">
+      <c r="B6" s="82"/>
+      <c r="C6" s="83"/>
+      <c r="D6" s="87">
         <f>AVERAGE('Process Summary'!I4:I33,'Project Tracker'!O2,'Project Tracker'!O7)</f>
-        <v>6.25E-2</v>
-      </c>
-      <c r="E6" s="59"/>
-      <c r="F6" s="60"/>
-      <c r="G6" s="65">
+        <v>4.8437500000000001E-2</v>
+      </c>
+      <c r="E6" s="88"/>
+      <c r="F6" s="89"/>
+      <c r="G6" s="94">
         <f>COUNTIF('Process Summary'!D4:D33,"Completed")</f>
         <v>0</v>
       </c>
-      <c r="H6" s="66"/>
-      <c r="I6" s="67"/>
-      <c r="J6" s="72">
+      <c r="H6" s="95"/>
+      <c r="I6" s="96"/>
+      <c r="J6" s="101">
         <f ca="1">COUNTIF('Process Summary'!J4:J33,"Red")</f>
         <v>4</v>
       </c>
-      <c r="K6" s="73"/>
-      <c r="L6" s="74"/>
+      <c r="K6" s="102"/>
+      <c r="L6" s="103"/>
       <c r="N6" s="13" t="s">
         <v>54</v>
       </c>
@@ -1872,39 +1915,39 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:15" ht="14.65" customHeight="1">
-      <c r="A7" s="52"/>
-      <c r="B7" s="53"/>
-      <c r="C7" s="54"/>
-      <c r="D7" s="58"/>
-      <c r="E7" s="59"/>
-      <c r="F7" s="60"/>
-      <c r="G7" s="65"/>
-      <c r="H7" s="66"/>
-      <c r="I7" s="67"/>
-      <c r="J7" s="72"/>
-      <c r="K7" s="73"/>
-      <c r="L7" s="74"/>
+    <row r="7" spans="1:15" ht="14.75" customHeight="1">
+      <c r="A7" s="81"/>
+      <c r="B7" s="82"/>
+      <c r="C7" s="83"/>
+      <c r="D7" s="87"/>
+      <c r="E7" s="88"/>
+      <c r="F7" s="89"/>
+      <c r="G7" s="94"/>
+      <c r="H7" s="95"/>
+      <c r="I7" s="96"/>
+      <c r="J7" s="101"/>
+      <c r="K7" s="102"/>
+      <c r="L7" s="103"/>
       <c r="N7" s="13"/>
       <c r="O7" s="13"/>
     </row>
-    <row r="8" spans="1:15" ht="14.65" customHeight="1">
-      <c r="A8" s="55"/>
-      <c r="B8" s="56"/>
-      <c r="C8" s="57"/>
-      <c r="D8" s="61"/>
-      <c r="E8" s="62"/>
-      <c r="F8" s="63"/>
-      <c r="G8" s="68"/>
-      <c r="H8" s="69"/>
-      <c r="I8" s="70"/>
-      <c r="J8" s="75"/>
-      <c r="K8" s="76"/>
-      <c r="L8" s="77"/>
+    <row r="8" spans="1:15" ht="14.75" customHeight="1">
+      <c r="A8" s="84"/>
+      <c r="B8" s="85"/>
+      <c r="C8" s="86"/>
+      <c r="D8" s="90"/>
+      <c r="E8" s="91"/>
+      <c r="F8" s="92"/>
+      <c r="G8" s="97"/>
+      <c r="H8" s="98"/>
+      <c r="I8" s="99"/>
+      <c r="J8" s="104"/>
+      <c r="K8" s="105"/>
+      <c r="L8" s="106"/>
       <c r="N8" s="13"/>
       <c r="O8" s="13"/>
     </row>
-    <row r="9" spans="1:15" ht="14.65" customHeight="1">
+    <row r="9" spans="1:15" ht="14.75" customHeight="1">
       <c r="A9" s="3"/>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
@@ -1920,85 +1963,85 @@
       <c r="N9" s="13"/>
       <c r="O9" s="13"/>
     </row>
-    <row r="10" spans="1:15" ht="14.65" customHeight="1">
-      <c r="A10" s="86" t="s">
+    <row r="10" spans="1:15" ht="14.75" customHeight="1">
+      <c r="A10" s="57" t="s">
         <v>79</v>
       </c>
-      <c r="B10" s="86"/>
-      <c r="C10" s="86"/>
-      <c r="D10" s="93" t="s">
+      <c r="B10" s="57"/>
+      <c r="C10" s="57"/>
+      <c r="D10" s="64" t="s">
         <v>80</v>
       </c>
-      <c r="E10" s="93"/>
-      <c r="F10" s="93"/>
-      <c r="G10" s="100" t="s">
+      <c r="E10" s="64"/>
+      <c r="F10" s="64"/>
+      <c r="G10" s="71" t="s">
         <v>81</v>
       </c>
-      <c r="H10" s="100"/>
-      <c r="I10" s="100"/>
-      <c r="J10" s="78" t="s">
+      <c r="H10" s="71"/>
+      <c r="I10" s="71"/>
+      <c r="J10" s="49" t="s">
         <v>82</v>
       </c>
-      <c r="K10" s="78"/>
-      <c r="L10" s="78"/>
+      <c r="K10" s="49"/>
+      <c r="L10" s="49"/>
       <c r="N10" s="13"/>
       <c r="O10" s="13"/>
     </row>
-    <row r="11" spans="1:15" ht="14.65" customHeight="1">
-      <c r="A11" s="87">
+    <row r="11" spans="1:15" ht="14.75" customHeight="1">
+      <c r="A11" s="58">
         <f>COUNTIF('Process Summary'!D4:D33,"In Progress")</f>
         <v>0</v>
       </c>
-      <c r="B11" s="88"/>
-      <c r="C11" s="89"/>
-      <c r="D11" s="94">
+      <c r="B11" s="59"/>
+      <c r="C11" s="60"/>
+      <c r="D11" s="65">
         <f>COUNTIF('Process Summary'!D4:D33,"Not Started")</f>
         <v>30</v>
       </c>
-      <c r="E11" s="95"/>
-      <c r="F11" s="96"/>
-      <c r="G11" s="101">
+      <c r="E11" s="66"/>
+      <c r="F11" s="67"/>
+      <c r="G11" s="72">
         <f>COUNTIF('Process Summary'!D4:D33,"On Hold")</f>
         <v>0</v>
       </c>
-      <c r="H11" s="102"/>
-      <c r="I11" s="103"/>
-      <c r="J11" s="79">
+      <c r="H11" s="73"/>
+      <c r="I11" s="74"/>
+      <c r="J11" s="50">
         <f ca="1">COUNTIF('Process Summary'!J4:J33,"Amber")</f>
         <v>0</v>
       </c>
-      <c r="K11" s="80"/>
-      <c r="L11" s="81"/>
-    </row>
-    <row r="12" spans="1:15" ht="14.65" customHeight="1">
-      <c r="A12" s="87"/>
-      <c r="B12" s="88"/>
-      <c r="C12" s="89"/>
-      <c r="D12" s="94"/>
-      <c r="E12" s="95"/>
-      <c r="F12" s="96"/>
-      <c r="G12" s="101"/>
-      <c r="H12" s="102"/>
-      <c r="I12" s="103"/>
-      <c r="J12" s="79"/>
-      <c r="K12" s="80"/>
-      <c r="L12" s="81"/>
-    </row>
-    <row r="13" spans="1:15" ht="14.65" customHeight="1">
-      <c r="A13" s="90"/>
-      <c r="B13" s="91"/>
-      <c r="C13" s="92"/>
-      <c r="D13" s="97"/>
-      <c r="E13" s="98"/>
-      <c r="F13" s="99"/>
-      <c r="G13" s="104"/>
-      <c r="H13" s="105"/>
-      <c r="I13" s="106"/>
-      <c r="J13" s="82"/>
-      <c r="K13" s="83"/>
-      <c r="L13" s="84"/>
-    </row>
-    <row r="14" spans="1:15" ht="14.65" customHeight="1">
+      <c r="K11" s="51"/>
+      <c r="L11" s="52"/>
+    </row>
+    <row r="12" spans="1:15" ht="14.75" customHeight="1">
+      <c r="A12" s="58"/>
+      <c r="B12" s="59"/>
+      <c r="C12" s="60"/>
+      <c r="D12" s="65"/>
+      <c r="E12" s="66"/>
+      <c r="F12" s="67"/>
+      <c r="G12" s="72"/>
+      <c r="H12" s="73"/>
+      <c r="I12" s="74"/>
+      <c r="J12" s="50"/>
+      <c r="K12" s="51"/>
+      <c r="L12" s="52"/>
+    </row>
+    <row r="13" spans="1:15" ht="14.75" customHeight="1">
+      <c r="A13" s="61"/>
+      <c r="B13" s="62"/>
+      <c r="C13" s="63"/>
+      <c r="D13" s="68"/>
+      <c r="E13" s="69"/>
+      <c r="F13" s="70"/>
+      <c r="G13" s="75"/>
+      <c r="H13" s="76"/>
+      <c r="I13" s="77"/>
+      <c r="J13" s="53"/>
+      <c r="K13" s="54"/>
+      <c r="L13" s="55"/>
+    </row>
+    <row r="14" spans="1:15" ht="14.75" customHeight="1">
       <c r="A14" s="31"/>
       <c r="B14" s="31"/>
       <c r="C14" s="31"/>
@@ -2012,7 +2055,7 @@
       <c r="K14" s="30"/>
       <c r="L14" s="30"/>
     </row>
-    <row r="15" spans="1:15" ht="14.65" customHeight="1">
+    <row r="15" spans="1:15" ht="14.75" customHeight="1">
       <c r="A15" s="3"/>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
@@ -2026,25 +2069,25 @@
       <c r="K15" s="3"/>
       <c r="L15" s="3"/>
     </row>
-    <row r="16" spans="1:15" ht="14.65" customHeight="1">
-      <c r="A16" s="85" t="s">
+    <row r="16" spans="1:15" ht="14.75" customHeight="1">
+      <c r="A16" s="56" t="s">
         <v>83</v>
       </c>
-      <c r="B16" s="85"/>
-      <c r="C16" s="85"/>
-      <c r="D16" s="85"/>
-      <c r="E16" s="85"/>
-      <c r="F16" s="85"/>
-      <c r="G16" s="85" t="s">
+      <c r="B16" s="56"/>
+      <c r="C16" s="56"/>
+      <c r="D16" s="56"/>
+      <c r="E16" s="56"/>
+      <c r="F16" s="56"/>
+      <c r="G16" s="56" t="s">
         <v>84</v>
       </c>
-      <c r="H16" s="85"/>
-      <c r="I16" s="85"/>
-      <c r="J16" s="85"/>
-      <c r="K16" s="85"/>
-      <c r="L16" s="85"/>
-    </row>
-    <row r="17" spans="1:12" ht="14.65" customHeight="1">
+      <c r="H16" s="56"/>
+      <c r="I16" s="56"/>
+      <c r="J16" s="56"/>
+      <c r="K16" s="56"/>
+      <c r="L16" s="56"/>
+    </row>
+    <row r="17" spans="1:12" ht="14.75" customHeight="1">
       <c r="A17" s="4" t="s">
         <v>85</v>
       </c>
@@ -2072,7 +2115,7 @@
       <c r="K17" s="3"/>
       <c r="L17" s="3"/>
     </row>
-    <row r="18" spans="1:12" ht="14.65" customHeight="1">
+    <row r="18" spans="1:12" ht="14.75" customHeight="1">
       <c r="A18" s="3" t="s">
         <v>89</v>
       </c>
@@ -2104,7 +2147,7 @@
       <c r="K18" s="3"/>
       <c r="L18" s="3"/>
     </row>
-    <row r="19" spans="1:12" ht="14.65" customHeight="1">
+    <row r="19" spans="1:12" ht="14.75" customHeight="1">
       <c r="A19" s="3" t="s">
         <v>91</v>
       </c>
@@ -2136,7 +2179,7 @@
       <c r="K19" s="3"/>
       <c r="L19" s="3"/>
     </row>
-    <row r="20" spans="1:12" ht="14.65" customHeight="1">
+    <row r="20" spans="1:12" ht="14.75" customHeight="1">
       <c r="A20" s="3" t="s">
         <v>93</v>
       </c>
@@ -2168,7 +2211,7 @@
       <c r="K20" s="3"/>
       <c r="L20" s="3"/>
     </row>
-    <row r="21" spans="1:12" ht="14.65" customHeight="1">
+    <row r="21" spans="1:12" ht="14.75" customHeight="1">
       <c r="A21" s="3" t="s">
         <v>95</v>
       </c>
@@ -2200,7 +2243,7 @@
       <c r="K21" s="3"/>
       <c r="L21" s="3"/>
     </row>
-    <row r="22" spans="1:12" ht="14.65" customHeight="1">
+    <row r="22" spans="1:12" ht="14.75" customHeight="1">
       <c r="A22" s="3" t="s">
         <v>97</v>
       </c>
@@ -2224,7 +2267,7 @@
       <c r="K22" s="3"/>
       <c r="L22" s="3"/>
     </row>
-    <row r="23" spans="1:12" ht="14.65" customHeight="1">
+    <row r="23" spans="1:12" ht="14.75" customHeight="1">
       <c r="A23" s="3" t="s">
         <v>98</v>
       </c>
@@ -2248,7 +2291,7 @@
       <c r="K23" s="3"/>
       <c r="L23" s="3"/>
     </row>
-    <row r="24" spans="1:12" ht="14.65" customHeight="1">
+    <row r="24" spans="1:12" ht="14.75" customHeight="1">
       <c r="A24" s="3"/>
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
@@ -2262,7 +2305,7 @@
       <c r="K24" s="3"/>
       <c r="L24" s="3"/>
     </row>
-    <row r="25" spans="1:12" ht="14.65" customHeight="1">
+    <row r="25" spans="1:12" ht="14.75" customHeight="1">
       <c r="A25" s="3"/>
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
@@ -2276,25 +2319,25 @@
       <c r="K25" s="3"/>
       <c r="L25" s="3"/>
     </row>
-    <row r="26" spans="1:12" ht="14.65" customHeight="1">
-      <c r="A26" s="85" t="s">
+    <row r="26" spans="1:12" ht="14.75" customHeight="1">
+      <c r="A26" s="56" t="s">
         <v>99</v>
       </c>
-      <c r="B26" s="85"/>
-      <c r="C26" s="85"/>
-      <c r="D26" s="85"/>
-      <c r="E26" s="85"/>
-      <c r="F26" s="85"/>
-      <c r="G26" s="85" t="s">
+      <c r="B26" s="56"/>
+      <c r="C26" s="56"/>
+      <c r="D26" s="56"/>
+      <c r="E26" s="56"/>
+      <c r="F26" s="56"/>
+      <c r="G26" s="56" t="s">
         <v>100</v>
       </c>
-      <c r="H26" s="85"/>
-      <c r="I26" s="85"/>
-      <c r="J26" s="85"/>
-      <c r="K26" s="85"/>
-      <c r="L26" s="85"/>
-    </row>
-    <row r="27" spans="1:12" ht="14.65" customHeight="1">
+      <c r="H26" s="56"/>
+      <c r="I26" s="56"/>
+      <c r="J26" s="56"/>
+      <c r="K26" s="56"/>
+      <c r="L26" s="56"/>
+    </row>
+    <row r="27" spans="1:12" ht="14.75" customHeight="1">
       <c r="A27" s="4" t="s">
         <v>2</v>
       </c>
@@ -2319,7 +2362,7 @@
       <c r="K27" s="3"/>
       <c r="L27" s="3"/>
     </row>
-    <row r="28" spans="1:12" ht="14.65" customHeight="1">
+    <row r="28" spans="1:12" ht="14.75" customHeight="1">
       <c r="A28" s="3" t="s">
         <v>47</v>
       </c>
@@ -2346,7 +2389,7 @@
       <c r="K28" s="3"/>
       <c r="L28" s="3"/>
     </row>
-    <row r="29" spans="1:12" ht="14.65" customHeight="1">
+    <row r="29" spans="1:12" ht="14.75" customHeight="1">
       <c r="A29" s="3" t="s">
         <v>51</v>
       </c>
@@ -2373,7 +2416,7 @@
       <c r="K29" s="3"/>
       <c r="L29" s="3"/>
     </row>
-    <row r="30" spans="1:12" ht="14.65" customHeight="1">
+    <row r="30" spans="1:12" ht="14.75" customHeight="1">
       <c r="A30" s="3" t="s">
         <v>55</v>
       </c>
@@ -2400,7 +2443,7 @@
       <c r="K30" s="3"/>
       <c r="L30" s="3"/>
     </row>
-    <row r="31" spans="1:12" ht="14.65" customHeight="1">
+    <row r="31" spans="1:12" ht="14.75" customHeight="1">
       <c r="A31" s="3" t="s">
         <v>59</v>
       </c>
@@ -2422,7 +2465,7 @@
       <c r="K31" s="3"/>
       <c r="L31" s="3"/>
     </row>
-    <row r="32" spans="1:12" ht="14.65" customHeight="1">
+    <row r="32" spans="1:12" ht="14.75" customHeight="1">
       <c r="A32" s="3"/>
       <c r="B32" s="3"/>
       <c r="C32" s="3"/>
@@ -2436,7 +2479,7 @@
       <c r="K32" s="3"/>
       <c r="L32" s="3"/>
     </row>
-    <row r="33" spans="1:12" ht="14.65" customHeight="1">
+    <row r="33" spans="1:12" ht="14.75" customHeight="1">
       <c r="A33" s="3"/>
       <c r="B33" s="3"/>
       <c r="C33" s="3"/>
@@ -2450,7 +2493,7 @@
       <c r="K33" s="3"/>
       <c r="L33" s="3"/>
     </row>
-    <row r="34" spans="1:12" ht="14.65" customHeight="1">
+    <row r="34" spans="1:12" ht="14.75" customHeight="1">
       <c r="A34" s="3"/>
       <c r="B34" s="3"/>
       <c r="C34" s="3"/>
@@ -2464,7 +2507,7 @@
       <c r="K34" s="3"/>
       <c r="L34" s="3"/>
     </row>
-    <row r="35" spans="1:12" ht="14.65" customHeight="1">
+    <row r="35" spans="1:12" ht="14.75" customHeight="1">
       <c r="A35" s="3"/>
       <c r="B35" s="3"/>
       <c r="C35" s="3"/>
@@ -2478,7 +2521,7 @@
       <c r="K35" s="3"/>
       <c r="L35" s="3"/>
     </row>
-    <row r="36" spans="1:12" ht="14.65" customHeight="1">
+    <row r="36" spans="1:12" ht="14.75" customHeight="1">
       <c r="A36" s="3"/>
       <c r="B36" s="3"/>
       <c r="C36" s="3"/>
@@ -2492,7 +2535,7 @@
       <c r="K36" s="3"/>
       <c r="L36" s="3"/>
     </row>
-    <row r="37" spans="1:12" ht="14.65" customHeight="1">
+    <row r="37" spans="1:12" ht="14.75" customHeight="1">
       <c r="A37" s="3"/>
       <c r="B37" s="3"/>
       <c r="C37" s="3"/>
@@ -2508,6 +2551,16 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="A1:L2"/>
+    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A6:C8"/>
+    <mergeCell ref="D5:F5"/>
+    <mergeCell ref="D6:F8"/>
+    <mergeCell ref="G5:I5"/>
+    <mergeCell ref="G6:I8"/>
+    <mergeCell ref="J5:L5"/>
+    <mergeCell ref="J6:L8"/>
     <mergeCell ref="J10:L10"/>
     <mergeCell ref="J11:L13"/>
     <mergeCell ref="A16:F16"/>
@@ -2520,16 +2573,6 @@
     <mergeCell ref="D11:F13"/>
     <mergeCell ref="G10:I10"/>
     <mergeCell ref="G11:I13"/>
-    <mergeCell ref="A1:L2"/>
-    <mergeCell ref="A3:L3"/>
-    <mergeCell ref="A5:C5"/>
-    <mergeCell ref="A6:C8"/>
-    <mergeCell ref="D5:F5"/>
-    <mergeCell ref="D6:F8"/>
-    <mergeCell ref="G5:I5"/>
-    <mergeCell ref="G6:I8"/>
-    <mergeCell ref="J5:L5"/>
-    <mergeCell ref="J6:L8"/>
   </mergeCells>
   <conditionalFormatting sqref="D18:D23">
     <cfRule type="dataBar" priority="1">
@@ -2576,16 +2619,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:J33"/>
-  <sheetFormatPr defaultRowHeight="14"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="50.58203125" style="16" customWidth="1"/>
+    <col min="1" max="1" width="50.5" style="16" customWidth="1"/>
     <col min="2" max="2" width="12.5" style="16" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.75" style="16" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.6640625" style="16" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10" style="16" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.75" style="16" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.6640625" style="16" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14.6640625" style="16" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.9140625" style="16" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.75" style="16" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" style="16" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.6640625" style="16" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="8.5" style="16" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="6.1640625" style="16" bestFit="1" customWidth="1"/>
     <col min="11" max="16384" width="8.6640625" style="16"/>
@@ -3815,34 +3858,34 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Z222"/>
-  <sheetFormatPr defaultRowHeight="21" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="21" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="13.6640625" style="16" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.1640625" style="16" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.1640625" style="16" customWidth="1"/>
-    <col min="4" max="4" width="21.4140625" style="16" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.08203125" style="16" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.75" style="16" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.08203125" style="16" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.4140625" style="16" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.08203125" style="16" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.08203125" style="16" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="33.25" style="16" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.83203125" style="16" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="16.1640625" style="16" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="13.75" style="16" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="13.83203125" style="16" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="10" style="16" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.25" style="16" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="17.83203125" style="16" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="19.1640625" style="16" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="18.6640625" style="16" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="11.5" style="16" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="11.9140625" style="16" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="20.58203125" style="16" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="16.08203125" style="16" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="15.9140625" style="16" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="14.83203125" style="16" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14" style="16" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="19.83203125" style="16" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.5" style="16" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.1640625" style="16" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.6640625" style="16" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.1640625" style="16" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.1640625" style="16" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12" style="16" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15" style="16" hidden="1" customWidth="1"/>
+    <col min="10" max="10" width="18" style="16" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="34" style="16" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.33203125" style="16" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.5" style="16" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="14.1640625" style="16" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14" style="16" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10.33203125" style="16" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.6640625" style="16" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="18.33203125" style="16" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="19.5" style="16" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="18.5" style="16" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="11.83203125" style="16" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="12.33203125" style="16" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="72.33203125" style="16" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="18.6640625" style="16" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="16.1640625" style="16" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="21.5" style="16" bestFit="1" customWidth="1"/>
     <col min="27" max="16384" width="8.6640625" style="16"/>
   </cols>
   <sheetData>
@@ -3985,13 +4028,17 @@
       <c r="D3" s="23" t="s">
         <v>168</v>
       </c>
-      <c r="E3" s="23"/>
+      <c r="E3" s="23" t="s">
+        <v>182</v>
+      </c>
       <c r="F3" s="23"/>
       <c r="G3" s="27"/>
       <c r="H3" s="21"/>
       <c r="I3" s="23"/>
       <c r="J3" s="23"/>
-      <c r="K3" s="23"/>
+      <c r="K3" s="23" t="s">
+        <v>178</v>
+      </c>
       <c r="L3" s="23"/>
       <c r="M3" s="23"/>
       <c r="N3" s="27" t="s">
@@ -4032,13 +4079,17 @@
       <c r="D4" s="23" t="s">
         <v>169</v>
       </c>
-      <c r="E4" s="23"/>
+      <c r="E4" s="23" t="s">
+        <v>182</v>
+      </c>
       <c r="F4" s="23"/>
       <c r="G4" s="23"/>
       <c r="H4" s="23"/>
       <c r="I4" s="23"/>
       <c r="J4" s="23"/>
-      <c r="K4" s="23"/>
+      <c r="K4" s="23" t="s">
+        <v>178</v>
+      </c>
       <c r="L4" s="23"/>
       <c r="M4" s="23"/>
       <c r="N4" s="27" t="s">
@@ -4077,16 +4128,28 @@
       <c r="B5" s="23"/>
       <c r="C5" s="23"/>
       <c r="D5" s="23" t="s">
-        <v>170</v>
-      </c>
-      <c r="E5" s="23"/>
-      <c r="F5" s="23"/>
+        <v>171</v>
+      </c>
+      <c r="E5" s="23" t="s">
+        <v>182</v>
+      </c>
+      <c r="F5" s="23" t="s">
+        <v>183</v>
+      </c>
       <c r="G5" s="27"/>
-      <c r="H5" s="21"/>
-      <c r="I5" s="47"/>
-      <c r="J5" s="47"/>
-      <c r="K5" s="23"/>
-      <c r="L5" s="23"/>
+      <c r="H5" s="21" t="s">
+        <v>184</v>
+      </c>
+      <c r="I5" s="27"/>
+      <c r="J5" s="23" t="s">
+        <v>183</v>
+      </c>
+      <c r="K5" s="23" t="s">
+        <v>178</v>
+      </c>
+      <c r="L5" s="23" t="s">
+        <v>185</v>
+      </c>
       <c r="M5" s="23"/>
       <c r="N5" s="27" t="s">
         <v>58</v>
@@ -4112,28 +4175,40 @@
         <v>Green</v>
       </c>
       <c r="V5" s="38" t="s">
-        <v>130</v>
-      </c>
-      <c r="W5" s="23"/>
-      <c r="X5" s="23"/>
-      <c r="Y5" s="23"/>
-      <c r="Z5" s="23"/>
+        <v>188</v>
+      </c>
+      <c r="W5" s="23" t="s">
+        <v>179</v>
+      </c>
+      <c r="X5" t="s">
+        <v>180</v>
+      </c>
+      <c r="Y5" s="25">
+        <v>46233</v>
+      </c>
+      <c r="Z5" s="23" t="s">
+        <v>181</v>
+      </c>
     </row>
     <row r="6" spans="1:26" ht="21" customHeight="1">
       <c r="A6" s="23"/>
       <c r="B6" s="23"/>
       <c r="C6" s="23"/>
       <c r="D6" s="23" t="s">
-        <v>171</v>
-      </c>
-      <c r="E6" s="23"/>
-      <c r="F6" s="23"/>
+        <v>170</v>
+      </c>
+      <c r="E6" s="23" t="s">
+        <v>182</v>
+      </c>
       <c r="G6" s="27"/>
-      <c r="H6" s="21"/>
-      <c r="I6" s="47"/>
-      <c r="J6" s="47"/>
-      <c r="K6" s="23"/>
-      <c r="L6" s="23"/>
+      <c r="H6" s="27"/>
+      <c r="I6" s="27"/>
+      <c r="J6" s="23" t="s">
+        <v>187</v>
+      </c>
+      <c r="K6" s="23" t="s">
+        <v>186</v>
+      </c>
       <c r="M6" s="23"/>
       <c r="N6" s="27" t="s">
         <v>58</v>
@@ -4184,13 +4259,12 @@
       <c r="K7" s="17"/>
       <c r="L7" s="17"/>
       <c r="M7" s="17"/>
-      <c r="N7" s="20" t="str">
-        <f>IF(O3=100%,"Completed",IF(N4="On Hold","On Hold",IF(N5="On Hold","On Hold",IF(N6="On Hold","On Hold",IF(N7="On Hold","On Hold",IF(N8="On Hold","On Hold",IF(N9="On Hold","On Hold",IF(O3&gt;0%,"In Progress","Not Started"))))))))</f>
-        <v>Completed</v>
+      <c r="N7" s="20" t="s">
+        <v>50</v>
       </c>
       <c r="O7" s="18">
-        <f>(O3*3+O4*5+O5+O6*IF(G2="LOW",13,IF(G2="MEDIUM",23,33)))/(9+IF(G2="LOW",13,IF(G2="MEDIUM",23,33)))</f>
-        <v>1</v>
+        <f>AVERAGE(O8:O11)</f>
+        <v>0.55000000000000004</v>
       </c>
       <c r="P7" s="19">
         <f>P8</f>
@@ -4204,11 +4278,11 @@
       <c r="S7" s="19"/>
       <c r="T7" s="48">
         <f ca="1">IF(N7="Cancelled","",IF(S7&lt;&gt;"",S7-Q7,IF(AND(N7&lt;&gt;"Completed",TODAY()&gt;Q7),TODAY()-Q7,0)))</f>
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="U7" s="17" t="str">
         <f t="shared" ref="U7:U11" ca="1" si="3">IF(N7="Cancelled","Gray",IF(N7="On Hold","Red",IF(N7="Completed",IF(T7&gt;5,"Red",IF(T7&gt;0,"Amber","Green")),IF(T7&gt;5,"Red",IF(T7&gt;0,"Amber","Green")))))</f>
-        <v>Green</v>
+        <v>Red</v>
       </c>
       <c r="V7" s="35" t="s">
         <v>130</v>
@@ -4225,13 +4299,17 @@
       <c r="D8" s="23" t="s">
         <v>168</v>
       </c>
-      <c r="E8" s="23"/>
+      <c r="E8" s="23" t="s">
+        <v>182</v>
+      </c>
       <c r="F8" s="23"/>
       <c r="G8" s="27"/>
       <c r="H8" s="21"/>
       <c r="I8" s="47"/>
       <c r="J8" s="47"/>
-      <c r="K8" s="23"/>
+      <c r="K8" s="23" t="s">
+        <v>178</v>
+      </c>
       <c r="L8" s="23"/>
       <c r="M8" s="23"/>
       <c r="N8" s="27" t="s">
@@ -4272,13 +4350,17 @@
       <c r="D9" s="23" t="s">
         <v>169</v>
       </c>
-      <c r="E9" s="23"/>
+      <c r="E9" s="23" t="s">
+        <v>182</v>
+      </c>
       <c r="F9" s="23"/>
       <c r="G9" s="27"/>
       <c r="H9" s="21"/>
       <c r="I9" s="47"/>
       <c r="J9" s="47"/>
-      <c r="K9" s="23"/>
+      <c r="K9" s="23" t="s">
+        <v>178</v>
+      </c>
       <c r="L9" s="23"/>
       <c r="M9" s="23"/>
       <c r="N9" s="27" t="s">
@@ -4317,23 +4399,32 @@
       <c r="B10" s="23"/>
       <c r="C10" s="23"/>
       <c r="D10" s="23" t="s">
-        <v>170</v>
-      </c>
-      <c r="E10" s="23"/>
-      <c r="F10" s="23"/>
+        <v>171</v>
+      </c>
+      <c r="E10" s="23" t="s">
+        <v>182</v>
+      </c>
+      <c r="F10" s="23" t="s">
+        <v>189</v>
+      </c>
       <c r="G10" s="27"/>
-      <c r="H10" s="21"/>
+      <c r="H10" s="21" t="s">
+        <v>184</v>
+      </c>
       <c r="I10" s="47"/>
-      <c r="J10" s="47"/>
-      <c r="K10" s="23"/>
+      <c r="J10" s="23" t="s">
+        <v>189</v>
+      </c>
+      <c r="K10" s="23" t="s">
+        <v>178</v>
+      </c>
       <c r="L10" s="23"/>
       <c r="M10" s="23"/>
       <c r="N10" s="27" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="O10" s="21">
-        <f t="shared" si="4"/>
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="P10" s="47">
         <v>46360</v>
@@ -4345,42 +4436,56 @@
       <c r="S10" s="23"/>
       <c r="T10" s="20">
         <f t="shared" ca="1" si="5"/>
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="U10" s="20" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Green</v>
+        <v>Red</v>
       </c>
       <c r="V10" s="38" t="s">
-        <v>130</v>
-      </c>
-      <c r="W10" s="23"/>
-      <c r="X10" s="23"/>
-      <c r="Y10" s="23"/>
-      <c r="Z10" s="23"/>
+        <v>188</v>
+      </c>
+      <c r="W10" t="s">
+        <v>190</v>
+      </c>
+      <c r="X10" t="s">
+        <v>180</v>
+      </c>
+      <c r="Y10" s="25">
+        <v>46233</v>
+      </c>
+      <c r="Z10" s="23" t="s">
+        <v>181</v>
+      </c>
     </row>
     <row r="11" spans="1:26" ht="21" customHeight="1">
       <c r="A11" s="23"/>
       <c r="B11" s="23"/>
       <c r="C11" s="23"/>
       <c r="D11" s="23" t="s">
-        <v>171</v>
-      </c>
-      <c r="E11" s="23"/>
+        <v>170</v>
+      </c>
+      <c r="E11" s="23" t="s">
+        <v>182</v>
+      </c>
       <c r="F11" s="23"/>
       <c r="G11" s="27"/>
       <c r="H11" s="21"/>
       <c r="I11" s="47"/>
-      <c r="J11" s="47"/>
-      <c r="K11" s="23"/>
+      <c r="J11" s="23" t="s">
+        <v>187</v>
+      </c>
+      <c r="K11" s="23" t="s">
+        <v>186</v>
+      </c>
       <c r="L11" s="23"/>
       <c r="M11" s="23"/>
       <c r="N11" s="27" t="s">
-        <v>58</v>
+        <v>11</v>
       </c>
       <c r="O11" s="21">
         <f t="shared" si="4"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P11" s="47">
         <v>46360</v>
@@ -4392,16 +4497,18 @@
       <c r="S11" s="23"/>
       <c r="T11" s="20">
         <f t="shared" ca="1" si="5"/>
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="U11" s="20" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>Green</v>
+        <v>Red</v>
       </c>
       <c r="V11" s="38" t="s">
         <v>130</v>
       </c>
-      <c r="W11" s="23"/>
+      <c r="W11" s="23" t="s">
+        <v>191</v>
+      </c>
       <c r="X11" s="23"/>
       <c r="Y11" s="23"/>
       <c r="Z11" s="23"/>
@@ -4540,7 +4647,7 @@
       </c>
       <c r="T13" s="17">
         <f t="shared" ref="T13:T76" ca="1" si="6">IF(N13="Cancelled","",IF(S13&lt;&gt;"",S13-Q13,IF(AND(N13&lt;&gt;"Completed",TODAY()&gt;Q13),TODAY()-Q13,0)))</f>
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="U13" s="17" t="str">
         <f t="shared" ref="U13:U76" ca="1" si="7">IF(N13="Cancelled","Gray",IF(N13="On Hold","Red",IF(N13="Completed",IF(T13&gt;5,"Red",IF(T13&gt;0,"Amber","Green")),IF(T13&gt;5,"Red",IF(T13&gt;0,"Amber","Green")))))</f>
@@ -4603,7 +4710,7 @@
       <c r="S14" s="28"/>
       <c r="T14" s="20">
         <f t="shared" ca="1" si="6"/>
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="U14" s="20" t="str">
         <f t="shared" ca="1" si="7"/>
@@ -4666,7 +4773,7 @@
       <c r="S15" s="28"/>
       <c r="T15" s="20">
         <f t="shared" ca="1" si="6"/>
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="U15" s="20" t="str">
         <f t="shared" ca="1" si="7"/>
@@ -4729,7 +4836,7 @@
       <c r="S16" s="28"/>
       <c r="T16" s="20">
         <f t="shared" ca="1" si="6"/>
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="U16" s="20" t="str">
         <f t="shared" ca="1" si="7"/>
@@ -4792,7 +4899,7 @@
       <c r="S17" s="28"/>
       <c r="T17" s="20">
         <f t="shared" ca="1" si="6"/>
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="U17" s="20" t="str">
         <f t="shared" ca="1" si="7"/>
@@ -4855,7 +4962,7 @@
       <c r="S18" s="28"/>
       <c r="T18" s="20">
         <f t="shared" ca="1" si="6"/>
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="U18" s="20" t="str">
         <f t="shared" ca="1" si="7"/>
@@ -4918,7 +5025,7 @@
       <c r="S19" s="28"/>
       <c r="T19" s="20">
         <f t="shared" ca="1" si="6"/>
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="U19" s="20" t="str">
         <f t="shared" ca="1" si="7"/>
@@ -4990,7 +5097,7 @@
       </c>
       <c r="T20" s="17">
         <f t="shared" ca="1" si="6"/>
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="U20" s="17" t="str">
         <f t="shared" ca="1" si="7"/>
@@ -5053,7 +5160,7 @@
       <c r="S21" s="28"/>
       <c r="T21" s="20">
         <f t="shared" ca="1" si="6"/>
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="U21" s="20" t="str">
         <f t="shared" ca="1" si="7"/>
@@ -5116,7 +5223,7 @@
       <c r="S22" s="28"/>
       <c r="T22" s="20">
         <f t="shared" ca="1" si="6"/>
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="U22" s="20" t="str">
         <f t="shared" ca="1" si="7"/>
@@ -5179,7 +5286,7 @@
       <c r="S23" s="28"/>
       <c r="T23" s="20">
         <f t="shared" ca="1" si="6"/>
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="U23" s="20" t="str">
         <f t="shared" ca="1" si="7"/>
@@ -5242,7 +5349,7 @@
       <c r="S24" s="28"/>
       <c r="T24" s="20">
         <f t="shared" ca="1" si="6"/>
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="U24" s="20" t="str">
         <f t="shared" ca="1" si="7"/>
@@ -5305,7 +5412,7 @@
       <c r="S25" s="28"/>
       <c r="T25" s="20">
         <f t="shared" ca="1" si="6"/>
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="U25" s="20" t="str">
         <f t="shared" ca="1" si="7"/>
@@ -5368,7 +5475,7 @@
       <c r="S26" s="28"/>
       <c r="T26" s="20">
         <f t="shared" ca="1" si="6"/>
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="U26" s="20" t="str">
         <f t="shared" ca="1" si="7"/>
@@ -5440,7 +5547,7 @@
       </c>
       <c r="T27" s="17">
         <f t="shared" ca="1" si="6"/>
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="U27" s="17" t="str">
         <f t="shared" ca="1" si="7"/>
@@ -5503,7 +5610,7 @@
       <c r="S28" s="28"/>
       <c r="T28" s="20">
         <f t="shared" ca="1" si="6"/>
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="U28" s="20" t="str">
         <f t="shared" ca="1" si="7"/>
@@ -5566,7 +5673,7 @@
       <c r="S29" s="28"/>
       <c r="T29" s="20">
         <f t="shared" ca="1" si="6"/>
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="U29" s="20" t="str">
         <f t="shared" ca="1" si="7"/>
@@ -5629,7 +5736,7 @@
       <c r="S30" s="28"/>
       <c r="T30" s="20">
         <f t="shared" ca="1" si="6"/>
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="U30" s="20" t="str">
         <f t="shared" ca="1" si="7"/>
@@ -5692,7 +5799,7 @@
       <c r="S31" s="28"/>
       <c r="T31" s="20">
         <f t="shared" ca="1" si="6"/>
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="U31" s="20" t="str">
         <f t="shared" ca="1" si="7"/>
@@ -5755,7 +5862,7 @@
       <c r="S32" s="28"/>
       <c r="T32" s="20">
         <f t="shared" ca="1" si="6"/>
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="U32" s="20" t="str">
         <f t="shared" ca="1" si="7"/>
@@ -5818,7 +5925,7 @@
       <c r="S33" s="28"/>
       <c r="T33" s="20">
         <f t="shared" ca="1" si="6"/>
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="U33" s="20" t="str">
         <f t="shared" ca="1" si="7"/>
@@ -5890,7 +5997,7 @@
       </c>
       <c r="T34" s="17">
         <f t="shared" ca="1" si="6"/>
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="U34" s="17" t="str">
         <f t="shared" ca="1" si="7"/>
@@ -5953,7 +6060,7 @@
       <c r="S35" s="28"/>
       <c r="T35" s="20">
         <f t="shared" ca="1" si="6"/>
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="U35" s="20" t="str">
         <f t="shared" ca="1" si="7"/>
@@ -6016,7 +6123,7 @@
       <c r="S36" s="28"/>
       <c r="T36" s="20">
         <f t="shared" ca="1" si="6"/>
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="U36" s="20" t="str">
         <f t="shared" ca="1" si="7"/>
@@ -6079,7 +6186,7 @@
       <c r="S37" s="28"/>
       <c r="T37" s="20">
         <f t="shared" ca="1" si="6"/>
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="U37" s="20" t="str">
         <f t="shared" ca="1" si="7"/>
@@ -6142,7 +6249,7 @@
       <c r="S38" s="28"/>
       <c r="T38" s="20">
         <f t="shared" ca="1" si="6"/>
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="U38" s="20" t="str">
         <f t="shared" ca="1" si="7"/>
@@ -6205,7 +6312,7 @@
       <c r="S39" s="28"/>
       <c r="T39" s="20">
         <f t="shared" ca="1" si="6"/>
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="U39" s="20" t="str">
         <f t="shared" ca="1" si="7"/>
@@ -6268,7 +6375,7 @@
       <c r="S40" s="28"/>
       <c r="T40" s="20">
         <f t="shared" ca="1" si="6"/>
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="U40" s="20" t="str">
         <f t="shared" ca="1" si="7"/>
@@ -6403,7 +6510,7 @@
       <c r="S42" s="28"/>
       <c r="T42" s="20">
         <f t="shared" ca="1" si="6"/>
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="U42" s="20" t="str">
         <f t="shared" ca="1" si="7"/>
@@ -6466,7 +6573,7 @@
       <c r="S43" s="28"/>
       <c r="T43" s="20">
         <f t="shared" ca="1" si="6"/>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="U43" s="20" t="str">
         <f t="shared" ca="1" si="7"/>
@@ -6529,7 +6636,7 @@
       <c r="S44" s="28"/>
       <c r="T44" s="20">
         <f t="shared" ca="1" si="6"/>
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="U44" s="20" t="str">
         <f t="shared" ca="1" si="7"/>
@@ -6853,7 +6960,7 @@
       <c r="S49" s="28"/>
       <c r="T49" s="20">
         <f t="shared" ca="1" si="6"/>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="U49" s="20" t="str">
         <f t="shared" ca="1" si="7"/>
@@ -6916,7 +7023,7 @@
       <c r="S50" s="28"/>
       <c r="T50" s="20">
         <f t="shared" ca="1" si="6"/>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="U50" s="20" t="str">
         <f t="shared" ca="1" si="7"/>
@@ -6979,11 +7086,11 @@
       <c r="S51" s="28"/>
       <c r="T51" s="20">
         <f t="shared" ca="1" si="6"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U51" s="20" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v>Green</v>
+        <v>Amber</v>
       </c>
       <c r="V51" s="38" t="s">
         <v>130</v>
@@ -7303,7 +7410,7 @@
       <c r="S56" s="28"/>
       <c r="T56" s="20">
         <f t="shared" ca="1" si="6"/>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="U56" s="20" t="str">
         <f t="shared" ca="1" si="7"/>
@@ -7366,7 +7473,7 @@
       <c r="S57" s="28"/>
       <c r="T57" s="20">
         <f t="shared" ca="1" si="6"/>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="U57" s="20" t="str">
         <f t="shared" ca="1" si="7"/>
@@ -7429,11 +7536,11 @@
       <c r="S58" s="28"/>
       <c r="T58" s="20">
         <f t="shared" ca="1" si="6"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U58" s="20" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v>Green</v>
+        <v>Amber</v>
       </c>
       <c r="V58" s="38" t="s">
         <v>130</v>
@@ -7753,7 +7860,7 @@
       <c r="S63" s="28"/>
       <c r="T63" s="20">
         <f t="shared" ca="1" si="6"/>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="U63" s="20" t="str">
         <f t="shared" ca="1" si="7"/>
@@ -7816,7 +7923,7 @@
       <c r="S64" s="28"/>
       <c r="T64" s="20">
         <f t="shared" ca="1" si="6"/>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="U64" s="20" t="str">
         <f t="shared" ca="1" si="7"/>
@@ -7879,11 +7986,11 @@
       <c r="S65" s="28"/>
       <c r="T65" s="20">
         <f t="shared" ca="1" si="6"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U65" s="20" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v>Green</v>
+        <v>Amber</v>
       </c>
       <c r="V65" s="38" t="s">
         <v>130</v>
@@ -17988,27 +18095,6 @@
     </row>
   </sheetData>
   <autoFilter ref="A12:Z222" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
-  <conditionalFormatting sqref="H5:H6 H3 H8:H11">
-    <cfRule type="dataBar" priority="43">
-      <dataBar>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FF5B9BD5"/>
-      </dataBar>
-    </cfRule>
-    <cfRule type="dataBar" priority="44">
-      <dataBar>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FF5B9BD5"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{EE540B03-4C84-4AD4-A414-502E5F8EF2F5}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="O2:O7">
     <cfRule type="dataBar" priority="21">
       <dataBar>
@@ -18100,8 +18186,29 @@
       <formula>U13="Gray"</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="H5 H3 H8:H11">
+    <cfRule type="dataBar" priority="45">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF5B9BD5"/>
+      </dataBar>
+    </cfRule>
+    <cfRule type="dataBar" priority="46">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF5B9BD5"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{EE540B03-4C84-4AD4-A414-502E5F8EF2F5}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="5">
-    <dataValidation type="list" sqref="N13:N222 G3 G5:G11 N2:N6 N8:N11" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" sqref="N13:N222 G3 N8:N11 N2:N6 G5:G11 H6:I6 I5" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Not Started,In Progress,On Hold,Completed,Cancelled"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="Z13:Z222" xr:uid="{2D62D783-F530-42BA-B632-A529B3310D65}">
@@ -18121,17 +18228,6 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{EE540B03-4C84-4AD4-A414-502E5F8EF2F5}">
-            <x14:dataBar>
-              <x14:cfvo type="min"/>
-              <x14:cfvo type="max"/>
-              <x14:negativeFillColor auto="1"/>
-              <x14:axisColor auto="1"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>H5:H6 H3 H8:H11</xm:sqref>
-        </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{75CBFE49-CFA1-42D4-81EE-DB4D77576ECC}">
             <x14:dataBar>
@@ -18165,6 +18261,17 @@
           </x14:cfRule>
           <xm:sqref>O13:O222</xm:sqref>
         </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{EE540B03-4C84-4AD4-A414-502E5F8EF2F5}">
+            <x14:dataBar>
+              <x14:cfvo type="min"/>
+              <x14:cfvo type="max"/>
+              <x14:negativeFillColor auto="1"/>
+              <x14:axisColor auto="1"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>H5 H3 H8:H11</xm:sqref>
+        </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
@@ -18173,7 +18280,7 @@
           <x14:formula1>
             <xm:f>Settings!$D$4:$D$8</xm:f>
           </x14:formula1>
-          <xm:sqref>N14:N19 N217:N222 N210:N215 N203:N208 N196:N201 N189:N194 N182:N187 N175:N180 N168:N173 N161:N166 N154:N159 N147:N152 N140:N145 N133:N138 N126:N131 N119:N124 N112:N117 N105:N110 N98:N103 N91:N96 N84:N89 N77:N82 N70:N75 N63:N68 N56:N61 N49:N54 N42:N47 N35:N40 N28:N33 N21:N26 G3 G5:G11 N3:N6 N8:N11</xm:sqref>
+          <xm:sqref>N14:N19 N217:N222 N210:N215 N203:N208 N196:N201 N189:N194 N182:N187 N175:N180 N168:N173 N161:N166 N154:N159 N147:N152 N140:N145 N133:N138 N126:N131 N119:N124 N112:N117 N105:N110 N98:N103 N91:N96 N84:N89 N77:N82 N70:N75 N63:N68 N56:N61 N49:N54 N42:N47 N35:N40 N28:N33 N21:N26 G3 N8:N11 N3:N6 G5:G11 H6:I6 I5</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -18184,12 +18291,12 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:H12"/>
-  <sheetFormatPr defaultRowHeight="14"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="8" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="20">
+    <row r="1" spans="1:8" ht="21">
       <c r="A1" s="108" t="s">
         <v>41</v>
       </c>

</xml_diff>